<commit_message>
feat: integrate wind farm models, hourly analytics and reusable skills
</commit_message>
<xml_diff>
--- a/风场数据/风电场.xlsx
+++ b/风场数据/风电场.xlsx
@@ -12,7 +12,8 @@
     <workbookView windowWidth="22096" windowHeight="9971"/>
   </bookViews>
   <sheets>
-    <sheet name="风机数据" sheetId="3" r:id="rId1"/>
+    <sheet name="风机参数" sheetId="4" r:id="rId1"/>
+    <sheet name="电量数据" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,12 +33,397 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
+  <si>
+    <t>项目</t>
+  </si>
+  <si>
+    <r>
+      <t>WTG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>7.5MW</t>
+    </r>
+  </si>
+  <si>
+    <t>叶轮</t>
+  </si>
+  <si>
+    <r>
+      <t>单机容量（M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>W</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
+    </r>
+  </si>
+  <si>
+    <t>叶片数</t>
+  </si>
+  <si>
+    <r>
+      <t>叶轮直径</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(m)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>扫风面积</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(m²)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>轮毂高度</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(m)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>切入风速</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>切出风速</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>20-25</t>
+  </si>
+  <si>
+    <t>发电机</t>
+  </si>
+  <si>
+    <t>型式</t>
+  </si>
+  <si>
+    <t>双馈</t>
+  </si>
+  <si>
+    <t>功率调节方式</t>
+  </si>
+  <si>
+    <t>变桨变速</t>
+  </si>
+  <si>
+    <t>变桨系统</t>
+  </si>
+  <si>
+    <t>独立</t>
+  </si>
+  <si>
+    <r>
+      <t>额定功率</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(kW)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>变频器输出电压</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(kV)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>变频器频率</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(Hz)</t>
+    </r>
+  </si>
+  <si>
+    <t>远程控制系统</t>
+  </si>
+  <si>
+    <t>SCADA</t>
+  </si>
+  <si>
+    <t>适合风区</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <r>
+      <t>极限生存风速（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>秒最大值</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/m/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>运行环境温度</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>℃</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>-30~+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>40</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>生存环境温度</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>℃</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>-40~+50</t>
+  </si>
   <si>
     <t>风机编号</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>X</t>
     </r>
     <r>
@@ -70,6 +456,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>Y</t>
     </r>
     <r>
@@ -555,7 +947,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -574,6 +966,69 @@
         <color auto="1"/>
       </top>
       <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -702,7 +1157,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -714,34 +1169,34 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -826,7 +1281,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -837,6 +1292,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1372,6 +1851,207 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr defaultColWidth="8.88073394495413" defaultRowHeight="14.5" outlineLevelCol="2"/>
+  <cols>
+    <col min="2" max="2" width="17.1009174311927" customWidth="1"/>
+    <col min="3" max="3" width="28.2018348623853" customWidth="1"/>
+    <col min="4" max="4" width="20.9816513761468" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.25" spans="1:3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="15.25" spans="1:3">
+      <c r="A2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="5">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="3" ht="15.25" spans="1:3">
+      <c r="A3" s="6"/>
+      <c r="B3" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="15.25" spans="1:3">
+      <c r="A4" s="6"/>
+      <c r="B4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="9">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="5" ht="15.25" spans="1:3">
+      <c r="A5" s="6"/>
+      <c r="B5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="9">
+        <v>38013</v>
+      </c>
+    </row>
+    <row r="6" ht="15.25" spans="1:3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="9">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" ht="15.25" spans="1:3">
+      <c r="A7" s="6"/>
+      <c r="B7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="9">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="8" ht="15.25" spans="1:3">
+      <c r="A8" s="10"/>
+      <c r="B8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="15.25" spans="1:3">
+      <c r="A9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" ht="15.25" spans="1:3">
+      <c r="A10" s="6"/>
+      <c r="B10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" ht="15.25" spans="1:3">
+      <c r="A11" s="6"/>
+      <c r="B11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" ht="15.25" spans="1:3">
+      <c r="A12" s="6"/>
+      <c r="B12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="9">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="13" ht="26.15" spans="1:3">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="9">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="14" ht="15.25" spans="1:3">
+      <c r="A14" s="6"/>
+      <c r="B14" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" ht="15.25" spans="1:3">
+      <c r="A15" s="10"/>
+      <c r="B15" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" ht="15.25" spans="1:3">
+      <c r="A16" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" ht="15.25" spans="1:3">
+      <c r="A17" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="9">
+        <v>59.5</v>
+      </c>
+    </row>
+    <row r="18" ht="15.25" spans="1:3">
+      <c r="A18" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" ht="15.25" spans="1:3">
+      <c r="A19" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="8.88073394495413" defaultRowHeight="14.5"/>
   <cols>
@@ -1382,42 +2062,42 @@
   <sheetData>
     <row r="1" ht="37.8" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2">
         <v>38397196</v>
@@ -1452,7 +2132,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2">
         <v>38394755</v>
@@ -1487,7 +2167,7 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B4" s="2">
         <v>38394357</v>
@@ -1522,7 +2202,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2">
         <v>38395523</v>
@@ -1557,7 +2237,7 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2">
         <v>38393046</v>
@@ -1592,7 +2272,7 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B7" s="2">
         <v>38396442</v>
@@ -1627,7 +2307,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B8" s="2">
         <v>38396420</v>
@@ -1662,7 +2342,7 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="B9" s="2">
         <v>38392412</v>
@@ -1697,10 +2377,10 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:11">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -1726,31 +2406,31 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:11">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H11" s="2">
         <v>167346.4</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="J11" s="2">
         <v>125509.8</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>